<commit_message>
Updating hydrogen_optimizer_v_0_3_2.py, adding canonical URL to <head>, adding images
</commit_message>
<xml_diff>
--- a/modelInputs/e_Hydrogen_LCA.xlsx
+++ b/modelInputs/e_Hydrogen_LCA.xlsx
@@ -12719,7 +12719,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>5.500550055005501e-06</v>
+        <v>6.074965068950853e-06</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -12790,7 +12790,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>0.002354235423542354</v>
+        <v>0.002600085049510965</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -12861,7 +12861,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2.354235423542354e-06</v>
+        <v>2.600085049510965e-06</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>2.537652417748341e-09</v>
+        <v>4.547211422595093e-09</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -13215,7 +13215,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>2.537652417748341e-09</v>
+        <v>4.547211422595093e-09</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>2.697879791404971e-05</v>
+        <v>4.834322351817748e-05</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13367,7 +13367,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>2.697879791404971e-05</v>
+        <v>4.834322351817748e-05</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -13443,7 +13443,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>4.107768705271929e-13</v>
+        <v>1.318961149121546e-12</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -13722,7 +13722,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>9.787282025625589e-07</v>
+        <v>6.776255707762564e-07</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -13793,7 +13793,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>76.14049586776865</v>
+        <v>50</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -13864,7 +13864,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>6.85950413223135</v>
+        <v>0</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>5.845920606040443e-05</v>
+        <v>0</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Changing new logo on multiple files
</commit_message>
<xml_diff>
--- a/modelInputs/e_Hydrogen_LCA.xlsx
+++ b/modelInputs/e_Hydrogen_LCA.xlsx
@@ -12719,7 +12719,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>5.778008898133703e-06</v>
+        <v>6.415191172696946e-06</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -12790,7 +12790,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>0.002472987808401225</v>
+        <v>0.002745701821914293</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -12861,7 +12861,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2.472987808401225e-06</v>
+        <v>2.745701821914293e-06</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>6.13704010555709e-09</v>
+        <v>3.179144810046098e-09</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -13215,7 +13215,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>6.13704010555709e-09</v>
+        <v>3.179144810046098e-09</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>6.524532817821964e-05</v>
+        <v>3.379876013352408e-05</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13367,7 +13367,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>6.524532817821964e-05</v>
+        <v>3.379876013352408e-05</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -13443,7 +13443,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>2.402479174379808e-12</v>
+        <v>6.447069171869162e-13</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -13722,7 +13722,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>6.584474885844729e-07</v>
+        <v>7.251141552511395e-07</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Updating requirements.txt and fixing issues in the main code
</commit_message>
<xml_diff>
--- a/modelInputs/e_Hydrogen_LCA.xlsx
+++ b/modelInputs/e_Hydrogen_LCA.xlsx
@@ -12719,7 +12719,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>6.415191172696946e-06</v>
+        <v>9.521089212605923e-06</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -12790,7 +12790,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>0.002745701821914293</v>
+        <v>0.004075026182995335</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -12861,7 +12861,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2.745701821914293e-06</v>
+        <v>4.075026182995335e-06</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13139,7 +13139,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>3.179144810046098e-09</v>
+        <v>2.881138625984989e-09</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -13215,7 +13215,7 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>3.179144810046098e-09</v>
+        <v>2.881138625984989e-09</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -13291,7 +13291,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>3.379876013352408e-05</v>
+        <v>3.063053718829681e-05</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13367,7 +13367,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>3.379876013352408e-05</v>
+        <v>3.063053718829681e-05</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -13443,7 +13443,7 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>6.447069171869162e-13</v>
+        <v>5.295049429672296e-13</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -13722,7 +13722,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>7.251141552511395e-07</v>
+        <v>7.351985906176993e-07</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -13793,7 +13793,7 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>50</v>
+        <v>34.56159148952512</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -13864,7 +13864,7 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>15.43840851047488</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>0</v>
+        <v>0.0001171893372134601</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>

</xml_diff>